<commit_message>
Trotter mesh: PO-0 and 3-roll order move to the week of 9/28
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WMbR8uWBiFLctZQqB3wnd7
</commit_message>
<xml_diff>
--- a/Mesh cutting supplier (Trotter)/Mesh_Maths_Production.xlsx
+++ b/Mesh cutting supplier (Trotter)/Mesh_Maths_Production.xlsx
@@ -535,7 +535,7 @@
     <t xml:space="preserve">OPEN PO AT FORECAST START — "PO-0" (released before the horizon begins)</t>
   </si>
   <si>
-    <t xml:space="preserve">ASSUMPTION: PO-0 goes out today, 9/24 — Trotter is onboarded. Move the date if it slips.</t>
+    <t xml:space="preserve">PO-0 and the 3-roll order go out the week of 9/28 (decided 9/24).</t>
   </si>
   <si>
     <t xml:space="preserve">PO-0 quantity (pieces)</t>
@@ -2643,8 +2643,8 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="str">
-        <f aca="false">"PO-0 released "&amp;TEXT($M$18,"m/d")&amp;" (roll must ship first, "&amp;$M$19&amp;" weeks) → pieces arrive week of "&amp;TEXT(INDEX($A$6:$A$31,$M$20),"m/d")&amp;". Stock runs out: "&amp;IF(MIN($U$6:$U$31)=0,"no stockout in the horizon","week of "&amp;TEXT(MIN($U$6:$U$31),"m/d")&amp;" (day level: out ~"&amp;TEXT(WORKDAY($M$18,INT(Inputs!B47/($M$7/5))),"ddd m/d")&amp;", PO-0 arrives ~"&amp;TEXT($M$28,"ddd m/d")&amp;") — ASK TROTTER TO SHIP PO-0 A FEW DAYS EARLY OR SHIP PARTIAL")&amp;". Later cut POs use rolls already at Trotter ("&amp;$M$13&amp;"-week lead time)."</f>
-        <v>PO-0 released 9/24 (roll must ship first, 4 weeks) → pieces arrive week of 10/26. Stock runs out: week of 10/19 (day level: out ~Tue 10/20, PO-0 arrives ~Tue 10/20) — ASK TROTTER TO SHIP PO-0 A FEW DAYS EARLY OR SHIP PARTIAL. Later cut POs use rolls already at Trotter (2-week lead time).</v>
+        <f aca="false">"PO-0 and 3 rolls ordered week of "&amp;TEXT($M$18,"m/d")&amp;" (roll must ship first, "&amp;$M$19&amp;" weeks) → pieces arrive week of "&amp;TEXT(INDEX($A$6:$A$31,$M$20),"m/d")&amp;". Stock runs out: "&amp;IF(MIN($U$6:$U$31)=0,"no stockout in the horizon","week of "&amp;TEXT(MIN($U$6:$U$31),"m/d")&amp;" (day level: out ~"&amp;TEXT(WORKDAY($M$5-1,INT($M$6/($M$7/5))+1),"ddd m/d")&amp;", PO-0 arrives ~"&amp;TEXT($M$28,"ddd m/d")&amp;") — ASK TROTTER TO SHIP PO-0 A FEW DAYS EARLY OR SHIP PARTIAL")&amp;". Later cut POs use rolls already at Trotter ("&amp;$M$13&amp;"-week lead time)."</f>
+        <v>PO-0 and 3 rolls ordered week of 9/28 (roll must ship first, 4 weeks) → pieces arrive week of 10/26. Stock runs out: week of 10/19 (day level: out ~Tue 10/20, PO-0 arrives ~Tue 10/20) — ASK TROTTER TO SHIP PO-0 A FEW DAYS EARLY OR SHIP PARTIAL. Later cut POs use rolls already at Trotter (2-week lead time).</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="M18" s="27" t="n">
         <f aca="false">Inputs!B55</f>
-        <v>46289</v>
+        <v>46293</v>
       </c>
       <c r="N18" s="18" t="s">
         <v>35</v>
@@ -4948,7 +4948,7 @@
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="48" t="str">
         <f aca="false">"• Physical count "&amp;TEXT(Inputs!B42,"m/d")&amp;": "&amp;TEXT(Inputs!B47,"#,##0")&amp;" pcs ("&amp;Inputs!B43&amp;" loose + "&amp;Inputs!B44&amp;" boxes) — "&amp;IF(Inputs!B47&lt;'Order Cadence'!B16,"BELOW the "&amp;TEXT('Order Cadence'!B16,"#,##0")&amp;" reorder point → release PO-0 now; ~"&amp;TEXT(Inputs!B60,"0.0")&amp;" days of cover left when it lands "&amp;TEXT(Inputs!B57,"m/d")&amp;" at the standard turnaround → ask Trotter to expedite it","above the reorder point")</f>
-        <v>• Physical count 9/24: 937 pcs (70 loose + 2 boxes) — BELOW the 1,000 reorder point → release PO-0 now; ~1.7 days of cover left when it lands 10/19 at the standard turnaround → ask Trotter to expedite it</v>
+        <v>• Physical count 9/24: 937 pcs (70 loose + 2 boxes) — BELOW the 1,000 reorder point → release PO-0 now; ~0.7 days of cover left when it lands 10/20 at the standard turnaround → ask Trotter to expedite it</v>
       </c>
       <c r="B34" s="48"/>
       <c r="C34" s="48"/>
@@ -5469,7 +5469,7 @@
         <v>34</v>
       </c>
       <c r="B55" s="60" t="n">
-        <v>46289</v>
+        <v>46293</v>
       </c>
       <c r="D55" s="59" t="s">
         <v>168</v>
@@ -5492,11 +5492,11 @@
       </c>
       <c r="B57" s="63" t="n">
         <f aca="false">IF(B56&lt;=0,"",'PO Schedule'!G14)</f>
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="D57" s="64" t="str">
         <f aca="false">"Calendar-day total says "&amp;TEXT(B55+B30,"m/d")&amp;"; rolling each leg off weekends pushes it to the date shown (release Thu 9/24 → roll due Sun → cut ends Wed → receive Sat → shelf Mon)"</f>
-        <v>Calendar-day total says 10/14; rolling each leg off weekends pushes it to the date shown (release Thu 9/24 → roll due Sun → cut ends Wed → receive Sat → shelf Mon)</v>
+        <v>Calendar-day total says 10/18; rolling each leg off weekends pushes it to the date shown (release Thu 9/24 → roll due Sun → cut ends Wed → receive Sat → shelf Mon)</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5517,7 +5517,7 @@
       </c>
       <c r="B59" s="52" t="n">
         <f aca="false">IF(B56&lt;=0,"n/a",B47-NETWORKDAYS(B42,B57-1)*B26/5)</f>
-        <v>87</v>
+        <v>37</v>
       </c>
       <c r="D59" s="57" t="s">
         <v>175</v>
@@ -5529,7 +5529,7 @@
       </c>
       <c r="B60" s="65" t="n">
         <f aca="false">IF(B56&lt;=0,"n/a",B59/(B26/5))</f>
-        <v>1.74</v>
+        <v>0.74</v>
       </c>
       <c r="D60" s="62" t="str">
         <f aca="false">IF(B56&lt;=0,"",IF(B60&lt;5,"⚠ Under a week of cover when the first roll lands — ask Trotter to cut PO-0 in the first available slot, not the full 2-week queue (their 1-day cut makes it realistic)","OK"))</f>
@@ -6956,27 +6956,27 @@
       </c>
       <c r="B14" s="95" t="n">
         <f aca="false">IF(Inputs!$B$56&gt;0,Inputs!$B$55,"")</f>
-        <v>46289</v>
+        <v>46293</v>
       </c>
       <c r="C14" s="95" t="n">
         <f aca="false">IF($B14="","",WORKDAY($B14+'Cycle Time'!$F$14-1,1))</f>
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="D14" s="95" t="n">
         <f aca="false">IF($B14="","",WORKDAY(C14+'Cycle Time'!$F$19-1,1))</f>
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="E14" s="96" t="n">
         <f aca="false">IF($B14="","",WORKDAY(D14+'Cycle Time'!$F$24-1,1))</f>
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="F14" s="95" t="n">
         <f aca="false">IF($B14="","",WORKDAY(E14+'Cycle Time'!$F$27-1,1))</f>
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="G14" s="95" t="n">
         <f aca="false">IF($B14="","",WORKDAY(F14+'Cycle Time'!$F$28-1,1))</f>
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="H14" s="97" t="n">
         <f aca="false">IF($B14="","",'6-Month Forecast'!$B$5+(Inputs!$B$58-1)*7)</f>
@@ -6988,23 +6988,23 @@
       </c>
       <c r="J14" s="56" t="n">
         <f aca="false">IF($B14="","",I14-$B14)</f>
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="K14" s="80" t="n">
         <f aca="false">IF($B14="","",I14-C14)</f>
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="L14" s="57" t="str">
         <f aca="false">IF($B14="","",IF(K14&gt;=$B$8,"Yes — "&amp;(K14-$B$8)&amp;" d margin","NO — short "&amp;($B$8-K14)&amp;" d"))</f>
-        <v>Yes — 4 d margin</v>
+        <v>Yes — 1 d margin</v>
       </c>
       <c r="M14" s="56" t="n">
         <f aca="false">IF($B14="","",I14-E14)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N14" s="61" t="n">
         <f aca="false">IF($B14="","",Inputs!$B$60)</f>
-        <v>1.74</v>
+        <v>0.74</v>
       </c>
       <c r="O14" s="57" t="str">
         <f aca="false">IF($B14="","",IF(SUMPRODUCT(($B$29:$B$32&lt;&gt;"")*($B$29:$B$32&lt;=E14)*($C$29:$C$32&gt;=C14))&gt;0,"⚠ holiday in window","clear"))</f>
@@ -8583,7 +8583,7 @@
       </c>
       <c r="D11" s="93" t="str">
         <f aca="false">"Released "&amp;TEXT(Inputs!B55,"m/d/yy")&amp;", credited to week "&amp;Inputs!B58&amp;" (arrives "&amp;TEXT(Inputs!B57,"m/d/yy")&amp;") — Inputs rows 54–61"</f>
-        <v>Released 9/24/26, credited to week 4 (arrives 10/19/26) — Inputs rows 54–61</v>
+        <v>Released 9/28/26, credited to week 4 (arrives 10/20/26) — Inputs rows 54–61</v>
       </c>
       <c r="E11" s="93"/>
       <c r="F11" s="93"/>

</xml_diff>

<commit_message>
Trotter mesh: rolls ordered two at a time
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WMbR8uWBiFLctZQqB3wnd7
</commit_message>
<xml_diff>
--- a/Mesh cutting supplier (Trotter)/Mesh_Maths_Production.xlsx
+++ b/Mesh cutting supplier (Trotter)/Mesh_Maths_Production.xlsx
@@ -118,7 +118,7 @@
     <t xml:space="preserve">Rolls per roll order</t>
   </si>
   <si>
-    <t xml:space="preserve">Equals the storage limit; ordered when the last roll at Trotter is committed</t>
+    <t xml:space="preserve">2 rolls per order (decided 9/24); Trotter can hold up to 3</t>
   </si>
   <si>
     <t xml:space="preserve">Trotter storage limit (rolls)</t>
@@ -151,7 +151,7 @@
     <t xml:space="preserve">Rolls ordered with PO-0</t>
   </si>
   <si>
-    <t xml:space="preserve">fills Trotter storage; 1 is cut for PO-0</t>
+    <t xml:space="preserve">2 rolls ship with PO-0; 1 is cut for PO-0</t>
   </si>
   <si>
     <t xml:space="preserve">Those rolls are at Trotter from week #</t>
@@ -2637,8 +2637,8 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="str">
-        <f aca="false">"Trotter stages in business days: material shipping "&amp;$M$24&amp;" → receiving "&amp;$M$25&amp;" → production "&amp;$M$26&amp;" (ships the same week; closed Fridays) → shipping to us "&amp;$M$27&amp;". 1 roll = "&amp;TEXT($M$8,"#,##0")&amp;" pcs · we use "&amp;TEXT($M$7,"#,##0")&amp;" pcs/week · we keep "&amp;$M$11&amp;" boxes ("&amp;TEXT($M$12,"#,##0")&amp;" pcs) as minimum stock · Trotter stores up to "&amp;$M$16&amp;" of our rolls, so rolls are ordered "&amp;$M$15&amp;" at a time."</f>
-        <v>Trotter stages in business days: material shipping 5 → receiving 5 → production 2 (ships the same week; closed Fridays) → shipping to us 5. 1 roll = 1,300 pcs · we use 250 pcs/week · we keep 2 boxes (867 pcs) as minimum stock · Trotter stores up to 3 of our rolls, so rolls are ordered 3 at a time.</v>
+        <f aca="false">"Trotter stages in business days: material shipping "&amp;$M$24&amp;" → receiving "&amp;$M$25&amp;" → production "&amp;$M$26&amp;" (ships the same week; closed Fridays) → shipping to us "&amp;$M$27&amp;". 1 roll = "&amp;TEXT($M$8,"#,##0")&amp;" pcs · we use "&amp;TEXT($M$7,"#,##0")&amp;" pcs/week · we keep "&amp;$M$11&amp;" boxes ("&amp;TEXT($M$12,"#,##0")&amp;" pcs) as minimum stock · Trotter stores up to "&amp;$M$16&amp;" of our rolls, and we ship "&amp;$M$15&amp;" rolls at a time."</f>
+        <v>Trotter stages in business days: material shipping 5 → receiving 5 → production 2 (ships the same week; closed Fridays) → shipping to us 5. 1 roll = 1,300 pcs · we use 250 pcs/week · we keep 2 boxes (867 pcs) as minimum stock · Trotter stores up to 3 of our rolls, and we ship 2 rolls at a time.</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2837,7 +2837,7 @@
       </c>
       <c r="G8" s="14" t="n">
         <f aca="false">G7-E7+IF(T8=$M$22,$M$21,0)+IF(T8&gt;$M$14,INDEX($H$6:H7,T8-$M$14),0)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H8" s="12" t="n">
         <f aca="false">IF(G8-E8+IF(T8&lt;$M$22,$M$21,0)+SUMPRODUCT(($T$6:T7&gt;T8-$M$14)*$H$6:H7)&lt;=0,$M$15,0)</f>
@@ -2897,7 +2897,7 @@
       </c>
       <c r="G9" s="14" t="n">
         <f aca="false">G8-E8+IF(T9=$M$22,$M$21,0)+IF(T9&gt;$M$14,INDEX($H$6:H8,T9-$M$14),0)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H9" s="12" t="n">
         <f aca="false">IF(G9-E9+IF(T9&lt;$M$22,$M$21,0)+SUMPRODUCT(($T$6:T8&gt;T9-$M$14)*$H$6:H8)&lt;=0,$M$15,0)</f>
@@ -2953,7 +2953,7 @@
       </c>
       <c r="G10" s="14" t="n">
         <f aca="false">G9-E9+IF(T10=$M$22,$M$21,0)+IF(T10&gt;$M$14,INDEX($H$6:H9,T10-$M$14),0)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H10" s="12" t="n">
         <f aca="false">IF(G10-E10+IF(T10&lt;$M$22,$M$21,0)+SUMPRODUCT(($T$6:T9&gt;T10-$M$14)*$H$6:H9)&lt;=0,$M$15,0)</f>
@@ -3010,7 +3010,7 @@
       </c>
       <c r="G11" s="14" t="n">
         <f aca="false">G10-E10+IF(T11=$M$22,$M$21,0)+IF(T11&gt;$M$14,INDEX($H$6:H10,T11-$M$14),0)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H11" s="12" t="n">
         <f aca="false">IF(G11-E11+IF(T11&lt;$M$22,$M$21,0)+SUMPRODUCT(($T$6:T10&gt;T11-$M$14)*$H$6:H10)&lt;=0,$M$15,0)</f>
@@ -3069,7 +3069,7 @@
       </c>
       <c r="G12" s="14" t="n">
         <f aca="false">G11-E11+IF(T12=$M$22,$M$21,0)+IF(T12&gt;$M$14,INDEX($H$6:H11,T12-$M$14),0)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H12" s="12" t="n">
         <f aca="false">IF(G12-E12+IF(T12&lt;$M$22,$M$21,0)+SUMPRODUCT(($T$6:T11&gt;T12-$M$14)*$H$6:H11)&lt;=0,$M$15,0)</f>
@@ -3126,7 +3126,7 @@
       </c>
       <c r="G13" s="14" t="n">
         <f aca="false">G12-E12+IF(T13=$M$22,$M$21,0)+IF(T13&gt;$M$14,INDEX($H$6:H12,T13-$M$14),0)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H13" s="12" t="n">
         <f aca="false">IF(G13-E13+IF(T13&lt;$M$22,$M$21,0)+SUMPRODUCT(($T$6:T12&gt;T13-$M$14)*$H$6:H12)&lt;=0,$M$15,0)</f>
@@ -3186,15 +3186,15 @@
       </c>
       <c r="G14" s="14" t="n">
         <f aca="false">G13-E13+IF(T14=$M$22,$M$21,0)+IF(T14&gt;$M$14,INDEX($H$6:H13,T14-$M$14),0)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H14" s="12" t="n">
         <f aca="false">IF(G14-E14+IF(T14&lt;$M$22,$M$21,0)+SUMPRODUCT(($T$6:T13&gt;T14-$M$14)*$H$6:H13)&lt;=0,$M$15,0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I14" s="15" t="str">
         <f aca="false">TRIM(IF(T14&lt;=$M$14,CHOOSE(MIN(T14,2),"Rolls shipping to Trotter (PO-0 order)","Trotter receiving our rolls"),"")&amp;" "&amp;IF(SUMPRODUCT(($T$6:T13&gt;=T14-$M$14)*($H$6:H13&gt;0)*(T14-$T$6:T13))=0,"",IF(SUMPRODUCT(($T$6:T13&gt;=T14-$M$14)*($H$6:H13&gt;0)*(T14-$T$6:T13))=$M$14,"Rolls received at Trotter","Rolls shipping to Trotter"))&amp;" "&amp;IF(H14&gt;0,"▲ ORDER "&amp;H14&amp;" ROLLS",""))</f>
-        <v/>
+        <v>▲ ORDER 2 ROLLS</v>
       </c>
       <c r="J14" s="16" t="str">
         <f aca="false">IF(D14&lt;0,"STOCKOUT",IF(D14&lt;$M$12,"below 2-box minimum",""))&amp;IF(G14&gt;$M$16," · storage &gt; "&amp;$M$16&amp;" rolls","")</f>
@@ -3246,7 +3246,7 @@
       </c>
       <c r="G15" s="14" t="n">
         <f aca="false">G14-E14+IF(T15=$M$22,$M$21,0)+IF(T15&gt;$M$14,INDEX($H$6:H14,T15-$M$14),0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H15" s="12" t="n">
         <f aca="false">IF(G15-E15+IF(T15&lt;$M$22,$M$21,0)+SUMPRODUCT(($T$6:T14&gt;T15-$M$14)*$H$6:H14)&lt;=0,$M$15,0)</f>
@@ -3254,7 +3254,7 @@
       </c>
       <c r="I15" s="15" t="str">
         <f aca="false">TRIM(IF(T15&lt;=$M$14,CHOOSE(MIN(T15,2),"Rolls shipping to Trotter (PO-0 order)","Trotter receiving our rolls"),"")&amp;" "&amp;IF(SUMPRODUCT(($T$6:T14&gt;=T15-$M$14)*($H$6:H14&gt;0)*(T15-$T$6:T14))=0,"",IF(SUMPRODUCT(($T$6:T14&gt;=T15-$M$14)*($H$6:H14&gt;0)*(T15-$T$6:T14))=$M$14,"Rolls received at Trotter","Rolls shipping to Trotter"))&amp;" "&amp;IF(H15&gt;0,"▲ ORDER "&amp;H15&amp;" ROLLS",""))</f>
-        <v/>
+        <v>Rolls shipping to Trotter</v>
       </c>
       <c r="J15" s="16" t="str">
         <f aca="false">IF(D15&lt;0,"STOCKOUT",IF(D15&lt;$M$12,"below 2-box minimum",""))&amp;IF(G15&gt;$M$16," · storage &gt; "&amp;$M$16&amp;" rolls","")</f>
@@ -3264,7 +3264,7 @@
         <v>28</v>
       </c>
       <c r="M15" s="21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N15" s="18" t="s">
         <v>29</v>
@@ -3305,7 +3305,7 @@
       </c>
       <c r="G16" s="14" t="n">
         <f aca="false">G15-E15+IF(T16=$M$22,$M$21,0)+IF(T16&gt;$M$14,INDEX($H$6:H15,T16-$M$14),0)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H16" s="12" t="n">
         <f aca="false">IF(G16-E16+IF(T16&lt;$M$22,$M$21,0)+SUMPRODUCT(($T$6:T15&gt;T16-$M$14)*$H$6:H15)&lt;=0,$M$15,0)</f>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="I16" s="15" t="str">
         <f aca="false">TRIM(IF(T16&lt;=$M$14,CHOOSE(MIN(T16,2),"Rolls shipping to Trotter (PO-0 order)","Trotter receiving our rolls"),"")&amp;" "&amp;IF(SUMPRODUCT(($T$6:T15&gt;=T16-$M$14)*($H$6:H15&gt;0)*(T16-$T$6:T15))=0,"",IF(SUMPRODUCT(($T$6:T15&gt;=T16-$M$14)*($H$6:H15&gt;0)*(T16-$T$6:T15))=$M$14,"Rolls received at Trotter","Rolls shipping to Trotter"))&amp;" "&amp;IF(H16&gt;0,"▲ ORDER "&amp;H16&amp;" ROLLS",""))</f>
-        <v/>
+        <v>Rolls received at Trotter</v>
       </c>
       <c r="J16" s="16" t="str">
         <f aca="false">IF(D16&lt;0,"STOCKOUT",IF(D16&lt;$M$12,"below 2-box minimum",""))&amp;IF(G16&gt;$M$16," · storage &gt; "&amp;$M$16&amp;" rolls","")</f>
@@ -3364,7 +3364,7 @@
       </c>
       <c r="G17" s="14" t="n">
         <f aca="false">G16-E16+IF(T17=$M$22,$M$21,0)+IF(T17&gt;$M$14,INDEX($H$6:H16,T17-$M$14),0)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H17" s="12" t="n">
         <f aca="false">IF(G17-E17+IF(T17&lt;$M$22,$M$21,0)+SUMPRODUCT(($T$6:T16&gt;T17-$M$14)*$H$6:H16)&lt;=0,$M$15,0)</f>
@@ -3424,7 +3424,7 @@
       </c>
       <c r="G18" s="14" t="n">
         <f aca="false">G17-E17+IF(T18=$M$22,$M$21,0)+IF(T18&gt;$M$14,INDEX($H$6:H17,T18-$M$14),0)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H18" s="12" t="n">
         <f aca="false">IF(G18-E18+IF(T18&lt;$M$22,$M$21,0)+SUMPRODUCT(($T$6:T17&gt;T18-$M$14)*$H$6:H17)&lt;=0,$M$15,0)</f>
@@ -3484,15 +3484,15 @@
       </c>
       <c r="G19" s="14" t="n">
         <f aca="false">G18-E18+IF(T19=$M$22,$M$21,0)+IF(T19&gt;$M$14,INDEX($H$6:H18,T19-$M$14),0)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H19" s="12" t="n">
         <f aca="false">IF(G19-E19+IF(T19&lt;$M$22,$M$21,0)+SUMPRODUCT(($T$6:T18&gt;T19-$M$14)*$H$6:H18)&lt;=0,$M$15,0)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I19" s="15" t="str">
         <f aca="false">TRIM(IF(T19&lt;=$M$14,CHOOSE(MIN(T19,2),"Rolls shipping to Trotter (PO-0 order)","Trotter receiving our rolls"),"")&amp;" "&amp;IF(SUMPRODUCT(($T$6:T18&gt;=T19-$M$14)*($H$6:H18&gt;0)*(T19-$T$6:T18))=0,"",IF(SUMPRODUCT(($T$6:T18&gt;=T19-$M$14)*($H$6:H18&gt;0)*(T19-$T$6:T18))=$M$14,"Rolls received at Trotter","Rolls shipping to Trotter"))&amp;" "&amp;IF(H19&gt;0,"▲ ORDER "&amp;H19&amp;" ROLLS",""))</f>
-        <v>▲ ORDER 3 ROLLS</v>
+        <v/>
       </c>
       <c r="J19" s="16" t="str">
         <f aca="false">IF(D19&lt;0,"STOCKOUT",IF(D19&lt;$M$12,"below 2-box minimum",""))&amp;IF(G19&gt;$M$16," · storage &gt; "&amp;$M$16&amp;" rolls","")</f>
@@ -3544,7 +3544,7 @@
       </c>
       <c r="G20" s="14" t="n">
         <f aca="false">G19-E19+IF(T20=$M$22,$M$21,0)+IF(T20&gt;$M$14,INDEX($H$6:H19,T20-$M$14),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H20" s="12" t="n">
         <f aca="false">IF(G20-E20+IF(T20&lt;$M$22,$M$21,0)+SUMPRODUCT(($T$6:T19&gt;T20-$M$14)*$H$6:H19)&lt;=0,$M$15,0)</f>
@@ -3552,7 +3552,7 @@
       </c>
       <c r="I20" s="15" t="str">
         <f aca="false">TRIM(IF(T20&lt;=$M$14,CHOOSE(MIN(T20,2),"Rolls shipping to Trotter (PO-0 order)","Trotter receiving our rolls"),"")&amp;" "&amp;IF(SUMPRODUCT(($T$6:T19&gt;=T20-$M$14)*($H$6:H19&gt;0)*(T20-$T$6:T19))=0,"",IF(SUMPRODUCT(($T$6:T19&gt;=T20-$M$14)*($H$6:H19&gt;0)*(T20-$T$6:T19))=$M$14,"Rolls received at Trotter","Rolls shipping to Trotter"))&amp;" "&amp;IF(H20&gt;0,"▲ ORDER "&amp;H20&amp;" ROLLS",""))</f>
-        <v>Rolls shipping to Trotter</v>
+        <v/>
       </c>
       <c r="J20" s="16" t="str">
         <f aca="false">IF(D20&lt;0,"STOCKOUT",IF(D20&lt;$M$12,"below 2-box minimum",""))&amp;IF(G20&gt;$M$16," · storage &gt; "&amp;$M$16&amp;" rolls","")</f>
@@ -3601,7 +3601,7 @@
       </c>
       <c r="G21" s="14" t="n">
         <f aca="false">G20-E20+IF(T21=$M$22,$M$21,0)+IF(T21&gt;$M$14,INDEX($H$6:H20,T21-$M$14),0)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H21" s="12" t="n">
         <f aca="false">IF(G21-E21+IF(T21&lt;$M$22,$M$21,0)+SUMPRODUCT(($T$6:T20&gt;T21-$M$14)*$H$6:H20)&lt;=0,$M$15,0)</f>
@@ -3609,7 +3609,7 @@
       </c>
       <c r="I21" s="15" t="str">
         <f aca="false">TRIM(IF(T21&lt;=$M$14,CHOOSE(MIN(T21,2),"Rolls shipping to Trotter (PO-0 order)","Trotter receiving our rolls"),"")&amp;" "&amp;IF(SUMPRODUCT(($T$6:T20&gt;=T21-$M$14)*($H$6:H20&gt;0)*(T21-$T$6:T20))=0,"",IF(SUMPRODUCT(($T$6:T20&gt;=T21-$M$14)*($H$6:H20&gt;0)*(T21-$T$6:T20))=$M$14,"Rolls received at Trotter","Rolls shipping to Trotter"))&amp;" "&amp;IF(H21&gt;0,"▲ ORDER "&amp;H21&amp;" ROLLS",""))</f>
-        <v>Rolls received at Trotter</v>
+        <v/>
       </c>
       <c r="J21" s="16" t="str">
         <f aca="false">IF(D21&lt;0,"STOCKOUT",IF(D21&lt;$M$12,"below 2-box minimum",""))&amp;IF(G21&gt;$M$16," · storage &gt; "&amp;$M$16&amp;" rolls","")</f>
@@ -3619,7 +3619,7 @@
         <v>39</v>
       </c>
       <c r="M21" s="21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N21" s="18" t="s">
         <v>40</v>
@@ -3660,7 +3660,7 @@
       </c>
       <c r="G22" s="14" t="n">
         <f aca="false">G21-E21+IF(T22=$M$22,$M$21,0)+IF(T22&gt;$M$14,INDEX($H$6:H21,T22-$M$14),0)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H22" s="12" t="n">
         <f aca="false">IF(G22-E22+IF(T22&lt;$M$22,$M$21,0)+SUMPRODUCT(($T$6:T21&gt;T22-$M$14)*$H$6:H21)&lt;=0,$M$15,0)</f>
@@ -3717,7 +3717,7 @@
       </c>
       <c r="G23" s="14" t="n">
         <f aca="false">G22-E22+IF(T23=$M$22,$M$21,0)+IF(T23&gt;$M$14,INDEX($H$6:H22,T23-$M$14),0)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H23" s="12" t="n">
         <f aca="false">IF(G23-E23+IF(T23&lt;$M$22,$M$21,0)+SUMPRODUCT(($T$6:T22&gt;T23-$M$14)*$H$6:H22)&lt;=0,$M$15,0)</f>
@@ -3771,15 +3771,15 @@
       </c>
       <c r="G24" s="14" t="n">
         <f aca="false">G23-E23+IF(T24=$M$22,$M$21,0)+IF(T24&gt;$M$14,INDEX($H$6:H23,T24-$M$14),0)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H24" s="12" t="n">
         <f aca="false">IF(G24-E24+IF(T24&lt;$M$22,$M$21,0)+SUMPRODUCT(($T$6:T23&gt;T24-$M$14)*$H$6:H23)&lt;=0,$M$15,0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I24" s="15" t="str">
         <f aca="false">TRIM(IF(T24&lt;=$M$14,CHOOSE(MIN(T24,2),"Rolls shipping to Trotter (PO-0 order)","Trotter receiving our rolls"),"")&amp;" "&amp;IF(SUMPRODUCT(($T$6:T23&gt;=T24-$M$14)*($H$6:H23&gt;0)*(T24-$T$6:T23))=0,"",IF(SUMPRODUCT(($T$6:T23&gt;=T24-$M$14)*($H$6:H23&gt;0)*(T24-$T$6:T23))=$M$14,"Rolls received at Trotter","Rolls shipping to Trotter"))&amp;" "&amp;IF(H24&gt;0,"▲ ORDER "&amp;H24&amp;" ROLLS",""))</f>
-        <v/>
+        <v>▲ ORDER 2 ROLLS</v>
       </c>
       <c r="J24" s="16" t="str">
         <f aca="false">IF(D24&lt;0,"STOCKOUT",IF(D24&lt;$M$12,"below 2-box minimum",""))&amp;IF(G24&gt;$M$16," · storage &gt; "&amp;$M$16&amp;" rolls","")</f>
@@ -3827,7 +3827,7 @@
       </c>
       <c r="G25" s="14" t="n">
         <f aca="false">G24-E24+IF(T25=$M$22,$M$21,0)+IF(T25&gt;$M$14,INDEX($H$6:H24,T25-$M$14),0)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H25" s="12" t="n">
         <f aca="false">IF(G25-E25+IF(T25&lt;$M$22,$M$21,0)+SUMPRODUCT(($T$6:T24&gt;T25-$M$14)*$H$6:H24)&lt;=0,$M$15,0)</f>
@@ -3835,7 +3835,7 @@
       </c>
       <c r="I25" s="15" t="str">
         <f aca="false">TRIM(IF(T25&lt;=$M$14,CHOOSE(MIN(T25,2),"Rolls shipping to Trotter (PO-0 order)","Trotter receiving our rolls"),"")&amp;" "&amp;IF(SUMPRODUCT(($T$6:T24&gt;=T25-$M$14)*($H$6:H24&gt;0)*(T25-$T$6:T24))=0,"",IF(SUMPRODUCT(($T$6:T24&gt;=T25-$M$14)*($H$6:H24&gt;0)*(T25-$T$6:T24))=$M$14,"Rolls received at Trotter","Rolls shipping to Trotter"))&amp;" "&amp;IF(H25&gt;0,"▲ ORDER "&amp;H25&amp;" ROLLS",""))</f>
-        <v/>
+        <v>Rolls shipping to Trotter</v>
       </c>
       <c r="J25" s="16" t="str">
         <f aca="false">IF(D25&lt;0,"STOCKOUT",IF(D25&lt;$M$12,"below 2-box minimum",""))&amp;IF(G25&gt;$M$16," · storage &gt; "&amp;$M$16&amp;" rolls","")</f>
@@ -3891,7 +3891,7 @@
       </c>
       <c r="I26" s="15" t="str">
         <f aca="false">TRIM(IF(T26&lt;=$M$14,CHOOSE(MIN(T26,2),"Rolls shipping to Trotter (PO-0 order)","Trotter receiving our rolls"),"")&amp;" "&amp;IF(SUMPRODUCT(($T$6:T25&gt;=T26-$M$14)*($H$6:H25&gt;0)*(T26-$T$6:T25))=0,"",IF(SUMPRODUCT(($T$6:T25&gt;=T26-$M$14)*($H$6:H25&gt;0)*(T26-$T$6:T25))=$M$14,"Rolls received at Trotter","Rolls shipping to Trotter"))&amp;" "&amp;IF(H26&gt;0,"▲ ORDER "&amp;H26&amp;" ROLLS",""))</f>
-        <v/>
+        <v>Rolls received at Trotter</v>
       </c>
       <c r="J26" s="16" t="str">
         <f aca="false">IF(D26&lt;0,"STOCKOUT",IF(D26&lt;$M$12,"below 2-box minimum",""))&amp;IF(G26&gt;$M$16," · storage &gt; "&amp;$M$16&amp;" rolls","")</f>

</xml_diff>